<commit_message>
toxicity calculation and code rearranged
adding documentation to code steps and calculating the toxicity using CA approach
</commit_message>
<xml_diff>
--- a/Docs/TaxoTox_output_template.xlsx
+++ b/Docs/TaxoTox_output_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\owner\Desktop\TaxoTox\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7585F68E-2510-41F9-B937-CBA73C147B0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37FF7158-B56E-471A-B51C-39D4AC1499AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="User-Input" sheetId="1" r:id="rId1"/>
@@ -641,12 +641,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D20"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.109375" customWidth="1"/>
+    <col min="1" max="1" width="20.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -660,97 +660,97 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>22</v>
       </c>
@@ -764,29 +764,30 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7143A302-7615-4E4C-9724-0D178ED03A28}">
   <dimension ref="A1:Q25"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.88671875" customWidth="1"/>
-    <col min="2" max="17" width="11.109375" style="2" customWidth="1"/>
+    <col min="1" max="1" width="12.85546875" customWidth="1"/>
+    <col min="2" max="5" width="11.140625" style="2" hidden="1" customWidth="1"/>
+    <col min="6" max="17" width="11.140625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B5" s="12" t="s">
         <v>44</v>
       </c>
@@ -812,7 +813,7 @@
       <c r="P5" s="13"/>
       <c r="Q5" s="14"/>
     </row>
-    <row r="6" spans="1:17" s="1" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:17" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
@@ -865,7 +866,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -886,7 +887,7 @@
       <c r="P7" s="7"/>
       <c r="Q7" s="8"/>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -907,7 +908,7 @@
       <c r="P8" s="7"/>
       <c r="Q8" s="8"/>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>6</v>
       </c>
@@ -928,7 +929,7 @@
       <c r="P9" s="7"/>
       <c r="Q9" s="8"/>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>7</v>
       </c>
@@ -949,7 +950,7 @@
       <c r="P10" s="7"/>
       <c r="Q10" s="8"/>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -970,7 +971,7 @@
       <c r="P11" s="7"/>
       <c r="Q11" s="8"/>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -991,7 +992,7 @@
       <c r="P12" s="7"/>
       <c r="Q12" s="8"/>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>10</v>
       </c>
@@ -1012,7 +1013,7 @@
       <c r="P13" s="7"/>
       <c r="Q13" s="8"/>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>11</v>
       </c>
@@ -1033,7 +1034,7 @@
       <c r="P14" s="7"/>
       <c r="Q14" s="8"/>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>12</v>
       </c>
@@ -1054,7 +1055,7 @@
       <c r="P15" s="7"/>
       <c r="Q15" s="8"/>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>13</v>
       </c>
@@ -1075,7 +1076,7 @@
       <c r="P16" s="7"/>
       <c r="Q16" s="8"/>
     </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>14</v>
       </c>
@@ -1096,7 +1097,7 @@
       <c r="P17" s="7"/>
       <c r="Q17" s="8"/>
     </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>15</v>
       </c>
@@ -1117,7 +1118,7 @@
       <c r="P18" s="7"/>
       <c r="Q18" s="8"/>
     </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>16</v>
       </c>
@@ -1138,7 +1139,7 @@
       <c r="P19" s="7"/>
       <c r="Q19" s="8"/>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>17</v>
       </c>
@@ -1159,7 +1160,7 @@
       <c r="P20" s="7"/>
       <c r="Q20" s="8"/>
     </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>18</v>
       </c>
@@ -1180,7 +1181,7 @@
       <c r="P21" s="7"/>
       <c r="Q21" s="8"/>
     </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>19</v>
       </c>
@@ -1201,7 +1202,7 @@
       <c r="P22" s="7"/>
       <c r="Q22" s="8"/>
     </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>20</v>
       </c>
@@ -1222,7 +1223,7 @@
       <c r="P23" s="7"/>
       <c r="Q23" s="8"/>
     </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>21</v>
       </c>
@@ -1243,7 +1244,7 @@
       <c r="P24" s="7"/>
       <c r="Q24" s="8"/>
     </row>
-    <row r="25" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>22</v>
       </c>
@@ -1278,29 +1279,30 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BEDFA2BB-C0B4-403F-9A34-24792199A470}">
   <dimension ref="A1:Q25"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.88671875" customWidth="1"/>
-    <col min="2" max="17" width="11.109375" style="2" customWidth="1"/>
+    <col min="1" max="1" width="12.85546875" customWidth="1"/>
+    <col min="2" max="5" width="11.140625" style="2" hidden="1" customWidth="1"/>
+    <col min="6" max="17" width="11.140625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B5" s="12" t="s">
         <v>26</v>
       </c>
@@ -1326,7 +1328,7 @@
       <c r="P5" s="13"/>
       <c r="Q5" s="14"/>
     </row>
-    <row r="6" spans="1:17" s="1" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:17" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
@@ -1379,7 +1381,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -1400,7 +1402,7 @@
       <c r="P7" s="7"/>
       <c r="Q7" s="8"/>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -1421,7 +1423,7 @@
       <c r="P8" s="7"/>
       <c r="Q8" s="8"/>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>6</v>
       </c>
@@ -1442,7 +1444,7 @@
       <c r="P9" s="7"/>
       <c r="Q9" s="8"/>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>7</v>
       </c>
@@ -1463,7 +1465,7 @@
       <c r="P10" s="7"/>
       <c r="Q10" s="8"/>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -1484,7 +1486,7 @@
       <c r="P11" s="7"/>
       <c r="Q11" s="8"/>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -1505,7 +1507,7 @@
       <c r="P12" s="7"/>
       <c r="Q12" s="8"/>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>10</v>
       </c>
@@ -1526,7 +1528,7 @@
       <c r="P13" s="7"/>
       <c r="Q13" s="8"/>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>11</v>
       </c>
@@ -1547,7 +1549,7 @@
       <c r="P14" s="7"/>
       <c r="Q14" s="8"/>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>12</v>
       </c>
@@ -1568,7 +1570,7 @@
       <c r="P15" s="7"/>
       <c r="Q15" s="8"/>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>13</v>
       </c>
@@ -1589,7 +1591,7 @@
       <c r="P16" s="7"/>
       <c r="Q16" s="8"/>
     </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>14</v>
       </c>
@@ -1610,7 +1612,7 @@
       <c r="P17" s="7"/>
       <c r="Q17" s="8"/>
     </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>15</v>
       </c>
@@ -1631,7 +1633,7 @@
       <c r="P18" s="7"/>
       <c r="Q18" s="8"/>
     </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>16</v>
       </c>
@@ -1652,7 +1654,7 @@
       <c r="P19" s="7"/>
       <c r="Q19" s="8"/>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>17</v>
       </c>
@@ -1673,7 +1675,7 @@
       <c r="P20" s="7"/>
       <c r="Q20" s="8"/>
     </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>18</v>
       </c>
@@ -1694,7 +1696,7 @@
       <c r="P21" s="7"/>
       <c r="Q21" s="8"/>
     </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>19</v>
       </c>
@@ -1715,7 +1717,7 @@
       <c r="P22" s="7"/>
       <c r="Q22" s="8"/>
     </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>20</v>
       </c>
@@ -1736,7 +1738,7 @@
       <c r="P23" s="7"/>
       <c r="Q23" s="8"/>
     </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>21</v>
       </c>
@@ -1757,7 +1759,7 @@
       <c r="P24" s="7"/>
       <c r="Q24" s="8"/>
     </row>
-    <row r="25" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>22</v>
       </c>
@@ -1792,29 +1794,30 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EF28DDE-9798-49F9-BBE2-2166A76E56D3}">
   <dimension ref="A1:Q25"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.88671875" customWidth="1"/>
-    <col min="2" max="17" width="11.109375" style="2" customWidth="1"/>
+    <col min="1" max="1" width="12.85546875" customWidth="1"/>
+    <col min="2" max="5" width="11.140625" style="2" hidden="1" customWidth="1"/>
+    <col min="6" max="17" width="11.140625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B5" s="12" t="s">
         <v>26</v>
       </c>
@@ -1840,7 +1843,7 @@
       <c r="P5" s="13"/>
       <c r="Q5" s="14"/>
     </row>
-    <row r="6" spans="1:17" s="1" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:17" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
@@ -1893,7 +1896,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -1914,7 +1917,7 @@
       <c r="P7" s="7"/>
       <c r="Q7" s="8"/>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -1935,7 +1938,7 @@
       <c r="P8" s="7"/>
       <c r="Q8" s="8"/>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>6</v>
       </c>
@@ -1956,7 +1959,7 @@
       <c r="P9" s="7"/>
       <c r="Q9" s="8"/>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>7</v>
       </c>
@@ -1977,7 +1980,7 @@
       <c r="P10" s="7"/>
       <c r="Q10" s="8"/>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -1998,7 +2001,7 @@
       <c r="P11" s="7"/>
       <c r="Q11" s="8"/>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -2019,7 +2022,7 @@
       <c r="P12" s="7"/>
       <c r="Q12" s="8"/>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>10</v>
       </c>
@@ -2040,7 +2043,7 @@
       <c r="P13" s="7"/>
       <c r="Q13" s="8"/>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>11</v>
       </c>
@@ -2061,7 +2064,7 @@
       <c r="P14" s="7"/>
       <c r="Q14" s="8"/>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>12</v>
       </c>
@@ -2082,7 +2085,7 @@
       <c r="P15" s="7"/>
       <c r="Q15" s="8"/>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>13</v>
       </c>
@@ -2103,7 +2106,7 @@
       <c r="P16" s="7"/>
       <c r="Q16" s="8"/>
     </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>14</v>
       </c>
@@ -2124,7 +2127,7 @@
       <c r="P17" s="7"/>
       <c r="Q17" s="8"/>
     </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>15</v>
       </c>
@@ -2145,7 +2148,7 @@
       <c r="P18" s="7"/>
       <c r="Q18" s="8"/>
     </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>16</v>
       </c>
@@ -2166,7 +2169,7 @@
       <c r="P19" s="7"/>
       <c r="Q19" s="8"/>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>17</v>
       </c>
@@ -2187,7 +2190,7 @@
       <c r="P20" s="7"/>
       <c r="Q20" s="8"/>
     </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>18</v>
       </c>
@@ -2208,7 +2211,7 @@
       <c r="P21" s="7"/>
       <c r="Q21" s="8"/>
     </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>19</v>
       </c>
@@ -2229,7 +2232,7 @@
       <c r="P22" s="7"/>
       <c r="Q22" s="8"/>
     </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>20</v>
       </c>
@@ -2250,7 +2253,7 @@
       <c r="P23" s="7"/>
       <c r="Q23" s="8"/>
     </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>21</v>
       </c>
@@ -2271,7 +2274,7 @@
       <c r="P24" s="7"/>
       <c r="Q24" s="8"/>
     </row>
-    <row r="25" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>22</v>
       </c>
@@ -2306,13 +2309,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9125011E-5109-4B74-B976-3737ED7F228A}">
   <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" customWidth="1"/>
-    <col min="2" max="5" width="14" style="2" customWidth="1"/>
+    <col min="1" max="1" width="12.5703125" customWidth="1"/>
+    <col min="2" max="2" width="14" style="2" hidden="1" customWidth="1"/>
+    <col min="3" max="5" width="14" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>38</v>
       </c>
@@ -2329,22 +2333,22 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>43</v>
       </c>

</xml_diff>